<commit_message>
Fix airborne finales and checkpoint controls before V157 release
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V157.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V157.xlsx
@@ -108,8 +108,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV157Table11" displayName="AuditV157Table11" ref="A5:E27" totalsRowShown="0">
-  <autoFilter ref="A5:E27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV157Table11" displayName="AuditV157Table11" ref="A5:E28" totalsRowShown="0">
+  <autoFilter ref="A5:E28"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V156"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Audit Excel V61 historique</t>
+          <t xml:space="preserve">Pont Excel V61/V63 et catalogue courant V62 ; audit V61 historique</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hash et comptes anciens seulement ; aucune revue fictive des 2 363 entités.</t>
+          <t xml:space="preserve">Classeur brut absent ; métadonnées du pont présentes (2363 entités globales, 2929 thématiques), 14 liens d’armes/3 de véhicules et catalogue jeu de 1329 entrées disponibles. Pas de revue du classeur brut.</t>
         </is>
       </c>
       <c r="E6" s="0">
@@ -1742,12 +1742,12 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a024ec81df0c045c9103f6e865d283386da6f0c88345faf2da516adf8ad67bc4</t>
+          <t xml:space="preserve">7d14f17fb8d9febb3276bc047ba72685241ae3c6e6028a6a828a20e7517e9764</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le rendu ajoute des appuis alternés bornés pour les sorties spatiales, sans modifier les quatre PNG sources.</t>
+          <t xml:space="preserve">Le rendu ajoute retombée visuelle et appuis alternés bornés ; la projection affine/caméra conserve les supports sans changer les PNG sources.</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
@@ -1769,12 +1769,12 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">03a482cc5097517f2c542d7784ba17dc0cf0d38ce61b6626c51cf2530b3281c4</t>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La sortie spatiale suit le verdict et son outro, conserve la caméra terminale et respecte pause/skip/mouvement réduit.</t>
+          <t xml:space="preserve">La retombée de rendu démarre au verdict réel, parallèlement aux phases admissibles au sol ; la sortie conserve caméra, pause, skip et mouvement réduit.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -1796,12 +1796,12 @@
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c029048154268a43019aef9914ed6a2d8002d0227e3470c18adbafc13d542550</t>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Une sortie de rendu séparée conserve les 40 séquences/200 clés historiques et ne modifie ni résultat ni coordonnées de combat.</t>
+          <t xml:space="preserve">Les retombées et sorties V157 ont leur propre identité de partie/tick ; les 40 séquences/200 clés historiques et les corps physiques restent inchangés.</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -1823,12 +1823,12 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1c14eb4d9e8cffe580abcfc6421a6d19c992bbe96fd2db4a17b5fc65e72b057e</t>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">L’interface rend les participants sortant vers les bords avec caméra fixe, en conservant l’accès au résultat.</t>
+          <t xml:space="preserve">L’interface présente la retombée vers le support puis la sortie vers les bords avec caméra fixe, sans modifier le résultat.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -1894,7 +1894,7 @@
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/forge-playtest-checkpoint-ui-v157.js</t>
+          <t xml:space="preserve">src/forge-editor-v130.css</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -1904,12 +1904,12 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">49064fe17a32e5875f2b6090718e87bb868f5e8015fac87cc7efe676bf367789</t>
+          <t xml:space="preserve">b645064e47bda9c8162f79ecdaa5a93aedd37a7f35fdaebb7e66bd6faed943de</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nouvelles commandes explicites Enregistrer/Reprendre/Effacer, avec message d’erreur et reprise du playtest courant.</t>
+          <t xml:space="preserve">Feuille de style nouvellement auditée : panneau checkpoint compact au-dessus du canvas et du HUD, repliable et accessible en 16:9 comme en viewport mobile.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -1921,7 +1921,7 @@
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/forge-playtest-checkpoint-v157.js</t>
+          <t xml:space="preserve">src/forge-playtest-checkpoint-ui-v157.js</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">16947f03cfe0b774d0cc78b9ed91993363b3727a11c0100241d8cd1add08c43f</t>
+          <t xml:space="preserve">9161d9152a551de3d60977a8f04610a8f1be6081affe1e906d32c492a96b15dd</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nouveau codec et stockage local bornés des checkpoints Forge, avec identité projet/équipement et refus avant mutation.</t>
+          <t xml:space="preserve">Nouvelles commandes explicites Enregistrer/Reprendre/Effacer accessibles en plein écran 16:9 et viewport mobile, avec erreurs et reprise du playtest courant.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -1948,7 +1948,7 @@
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-annex-registry-v87.js</t>
+          <t xml:space="preserve">src/forge-playtest-checkpoint-v157.js</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -1958,24 +1958,24 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">67d74d09b8ffed8f078516bf99259ee3491610947669f8acbb5616da3efbece7</t>
+          <t xml:space="preserve">d7930fd9d9056970e63e02d54b6e70a3a4a00de931c26c7551db59ee15b4569c</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Périmètre nouvellement audité : largeur de la zone animal-care accordée au sol et à sa nouvelle baie de service.</t>
+          <t xml:space="preserve">Nouveau codec et stockage local bornés des checkpoints Forge, avec identité projet/équipement/véhicule de départ et refus avant mutation.</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-annex-service-v157.mjs</t>
+          <t xml:space="preserve">scripts/verify-forge-playtest-checkpoint-v157.mjs</t>
         </is>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-furnishing-annex-revisions-v139.js</t>
+          <t xml:space="preserve">src/hub-annex-registry-v87.js</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8b189a9c9703fadf8ec93d979dfad1f429991237f476a96d068a932170a3e3b5</t>
+          <t xml:space="preserve">67d74d09b8ffed8f078516bf99259ee3491610947669f8acbb5616da3efbece7</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Périmètre nouvellement audité : mobilier de soins et séparation de service ajoutés hors couchages et enclos.</t>
+          <t xml:space="preserve">Périmètre nouvellement audité : largeur de la zone animal-care accordée au sol et à sa nouvelle baie de service.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
@@ -2002,7 +2002,7 @@
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-dressing-v134.js</t>
+          <t xml:space="preserve">src/hub-furnishing-annex-revisions-v139.js</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2012,12 +2012,12 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c1b5d8364ccf714ea64a540276197744537829d2524c0407c83b51adf822e8fd</t>
+          <t xml:space="preserve">8b189a9c9703fadf8ec93d979dfad1f429991237f476a96d068a932170a3e3b5</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Périmètre nouvellement audité : décoration de service animalier placée sur les supports de la salle agrandie.</t>
+          <t xml:space="preserve">Périmètre nouvellement audité : mobilier de soins et séparation de service ajoutés hors couchages et enclos.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-life-v136.js</t>
+          <t xml:space="preserve">src/hub-room-dressing-v134.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -2039,12 +2039,12 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">61c15a13031a7d25208a366d1e4f0975b71c317ae23edbf5493778f56f6fa05b</t>
+          <t xml:space="preserve">c1b5d8364ccf714ea64a540276197744537829d2524c0407c83b51adf822e8fd</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Périmètre nouvellement audité : accessoires muraux de service animalier cohérents avec les zones réservées.</t>
+          <t xml:space="preserve">Périmètre nouvellement audité : décoration de service animalier placée sur les supports de la salle agrandie.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -2056,7 +2056,7 @@
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/legacy-operations-v131.js</t>
+          <t xml:space="preserve">src/hub-room-life-v136.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -2066,24 +2066,24 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
+          <t xml:space="preserve">61c15a13031a7d25208a366d1e4f0975b71c317ae23edbf5493778f56f6fa05b</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Broodstorm conserve les explosifs déjà en vol lors d’une reprise, notamment le dernier dépensé avant checkpoint.</t>
+          <t xml:space="preserve">Périmètre nouvellement audité : accessoires muraux de service animalier cohérents avec les zones réservées.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-annex-service-v157.mjs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-life-v136.js</t>
+          <t xml:space="preserve">src/legacy-operations-v131.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -2093,24 +2093,24 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
+          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Périmètre nouvellement audité : cycle local de visite de service, avec retour au poste et priorités de routine préservées.</t>
+          <t xml:space="preserve">Broodstorm conserve les explosifs déjà en vol lors d’une reprise, notamment le dernier dépensé avant checkpoint.</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-annex-service-v157.mjs</t>
+          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/ship-animal-habitat-v87.js</t>
+          <t xml:space="preserve">src/npc-life-v136.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -2120,12 +2120,12 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">23b392916f7d76f89929e4e69e9b17c843cbd3784897893e7b49a33562ae26f4</t>
+          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Périmètre nouvellement audité : sol de l’accueil animalier étendu sans déplacer les six habitats existants.</t>
+          <t xml:space="preserve">Périmètre nouvellement audité : cycle local de visite de service, avec retour au poste et priorités de routine préservées.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -2137,25 +2137,52 @@
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/ship-animal-habitat-v87.js</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V156</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23b392916f7d76f89929e4e69e9b17c843cbd3784897893e7b49a33562ae26f4</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Périmètre nouvellement audité : sol de l’accueil animalier étendu sans déplacer les six habitats existants.</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-hub-annex-service-v157.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/special-operations-v131.js</t>
         </is>
       </c>
-      <c r="B27" s="0" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V156</t>
         </is>
       </c>
-      <c r="C27" s="0" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">30d8f872f1dafa1e379f56ea599d789ee2e8875e699034cda5934c7fcbbb35db</t>
         </is>
       </c>
-      <c r="D27" s="0" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Périmètre nouvellement audité : 21 accès jouables du registre actif V131, dont 20 adaptations partielles.</t>
         </is>
       </c>
-      <c r="E27" s="0" t="inlineStr">
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-operations-integration-v131.mjs</t>
         </is>
@@ -2257,17 +2284,17 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Après verdict et terminalV156 complets</t>
+          <t xml:space="preserve">Après phases de verdict admissibles ou retombée V157 autonome</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trajet de rendu vers bord ; appuis alternés ; caméra fixe</t>
+          <t xml:space="preserve">Retombée de rendu 180–600 ms si aérien ; puis trajet vers bord et appuis alternés</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rig natif admis seulement ; pas de marche dessinée complète ; pause/skip/mouvement réduit respectés.</t>
+          <t xml:space="preserve">Rig natif admis seulement ; corps physiques inchangés ; caméra fixe et appuis contrôlés ; pas de marche dessinée complète. Pause/skip/mouvement réduit respectés.</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
@@ -2295,17 +2322,17 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Après verdict et terminalV156 complets</t>
+          <t xml:space="preserve">Après phases de verdict admissibles ou retombée V157 autonome</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trajet de rendu vers bord ; appuis alternés ; caméra fixe</t>
+          <t xml:space="preserve">Retombée de rendu 180–600 ms si aérien ; puis trajet vers bord et appuis alternés</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rig natif admis seulement ; pas de marche dessinée complète ; pause/skip/mouvement réduit respectés.</t>
+          <t xml:space="preserve">Rig natif admis seulement ; corps physiques inchangés ; caméra fixe et appuis contrôlés ; pas de marche dessinée complète. Pause/skip/mouvement réduit respectés.</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
@@ -2333,17 +2360,17 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Après verdict et terminalV156 complets</t>
+          <t xml:space="preserve">Après phases de verdict admissibles ou retombée V157 autonome</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trajet de rendu vers bord ; appuis alternés ; caméra fixe</t>
+          <t xml:space="preserve">Retombée de rendu 180–600 ms si aérien ; puis trajet vers bord et appuis alternés</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rig natif admis seulement ; pas de marche dessinée complète ; pause/skip/mouvement réduit respectés.</t>
+          <t xml:space="preserve">Rig natif admis seulement ; corps physiques inchangés ; caméra fixe et appuis contrôlés ; pas de marche dessinée complète. Pause/skip/mouvement réduit respectés.</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
@@ -2371,17 +2398,17 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Après verdict et terminalV156 complets</t>
+          <t xml:space="preserve">Après phases de verdict admissibles ou retombée V157 autonome</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trajet de rendu vers bord ; appuis alternés ; caméra fixe</t>
+          <t xml:space="preserve">Retombée de rendu 180–600 ms si aérien ; puis trajet vers bord et appuis alternés</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rig natif admis seulement ; pas de marche dessinée complète ; pause/skip/mouvement réduit respectés.</t>
+          <t xml:space="preserve">Rig natif admis seulement ; corps physiques inchangés ; caméra fixe et appuis contrôlés ; pas de marche dessinée complète. Pause/skip/mouvement réduit respectés.</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
@@ -2583,7 +2610,7 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V157 ajoute après le verdict et l’outro une sortie de rendu vers les bords, avec appuis alternés bornés et caméra fixe. Corpus dessiné complet, audio et revue 1:1 restent ouverts.</t>
+          <t xml:space="preserve">V157 ajoute une retombée de rendu bornée si le verdict fige le rig en l’air, puis une sortie vers les bords. Corps physiques et verdict inchangés ; phases historiques au sol intactes. Dessins, audio et revue 1:1 restent ouverts.</t>
         </is>
       </c>
       <c r="G8" s="0">
@@ -2963,7 +2990,7 @@
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V157 ajoute après le verdict et l’outro une sortie de rendu vers les bords, avec appuis alternés bornés et caméra fixe. Corpus dessiné complet, audio et revue 1:1 restent ouverts.</t>
+          <t xml:space="preserve">V157 ajoute une retombée de rendu bornée si le verdict fige le rig en l’air, puis une sortie vers les bords. Corps physiques et verdict inchangés ; phases historiques au sol intactes. Dessins, audio et revue 1:1 restent ouverts.</t>
         </is>
       </c>
       <c r="G18" s="0">
@@ -3343,7 +3370,7 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V157 ajoute après le verdict et l’outro une sortie de rendu vers les bords, avec appuis alternés bornés et caméra fixe. Corpus dessiné complet, audio et revue 1:1 restent ouverts.</t>
+          <t xml:space="preserve">V157 ajoute une retombée de rendu bornée si le verdict fige le rig en l’air, puis une sortie vers les bords. Corps physiques et verdict inchangés ; phases historiques au sol intactes. Dessins, audio et revue 1:1 restent ouverts.</t>
         </is>
       </c>
       <c r="G28" s="0">
@@ -3723,7 +3750,7 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V157 ajoute après le verdict et l’outro une sortie de rendu vers les bords, avec appuis alternés bornés et caméra fixe. Corpus dessiné complet, audio et revue 1:1 restent ouverts.</t>
+          <t xml:space="preserve">V157 ajoute une retombée de rendu bornée si le verdict fige le rig en l’air, puis une sortie vers les bords. Corps physiques et verdict inchangés ; phases historiques au sol intactes. Dessins, audio et revue 1:1 restent ouverts.</t>
         </is>
       </c>
       <c r="G38" s="0">
@@ -8034,7 +8061,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un slot ; 4 Mio ; identité projet/équipement ; Enregistrer/Reprendre/Effacer ; validation avant mutation.</t>
+          <t xml:space="preserve">Un slot ; 4 Mio ; même projet/équipe/équipement/véhicule de départ ; commandes visibles en plein écran 16:9 et viewport mobile ; validation avant mutation.</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
@@ -8347,7 +8374,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sortie spatiale V157 séparée des 40 séquences/200 clés héritées.</t>
+          <t xml:space="preserve">Retombée et sortie de rendu V157 séparées des 40 séquences/200 clés héritées ; identités de partie/tick autonomes.</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -8548,7 +8575,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatre rigs, caméra fixe, appuis, fin du résultat et contrôles pause/skip/mouvement réduit.</t>
+          <t xml:space="preserve">Quatre rigs ; retombée de rendu monotone, affine/caméra et appuis ; deux aériens sans faux participant historique ; pause/skip/réduit et corps physiques intacts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preserve checkpoint action focus across asynchronous saves
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V157.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V157.xlsx
@@ -1931,12 +1931,12 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9161d9152a551de3d60977a8f04610a8f1be6081affe1e906d32c492a96b15dd</t>
+          <t xml:space="preserve">cfe79aa2a8a7e59fd667ba1ce25855afe1431d4bae93592a46cc5f4d6b97d2eb</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nouvelles commandes explicites Enregistrer/Reprendre/Effacer accessibles en plein écran 16:9 et viewport mobile, avec erreurs et reprise du playtest courant.</t>
+          <t xml:space="preserve">Commandes explicites accessibles en 16:9/mobile ; après action asynchrone, focus restitué seulement au contrôle initial du même moteur/session, sans voler un autre focus ni revenir après navigation.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -8061,7 +8061,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un slot ; 4 Mio ; même projet/équipe/équipement/véhicule de départ ; commandes visibles en plein écran 16:9 et viewport mobile ; validation avant mutation.</t>
+          <t xml:space="preserve">Un slot ; 4 Mio ; même projet/équipe/équipement/véhicule de départ ; commandes visibles en 16:9/mobile ; focus asynchrone gardé par moteur/session ; validation avant mutation.</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Keep keyboard focus inside checkpoint controls while saving
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V157.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V157.xlsx
@@ -1931,12 +1931,12 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfe79aa2a8a7e59fd667ba1ce25855afe1431d4bae93592a46cc5f4d6b97d2eb</t>
+          <t xml:space="preserve">85032efba0f8071afc69af9369682ce372c0ca6e718e6898c1ad456259ceafee</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commandes explicites accessibles en 16:9/mobile ; après action asynchrone, focus restitué seulement au contrôle initial du même moteur/session, sans voler un autre focus ni revenir après navigation.</t>
+          <t xml:space="preserve">Commandes accessibles en 16:9/mobile ; focus placé synchronement sur le résumé avant désactivation, puis restitué sous gardes moteur/session sans voler un autre focus ni revenir après navigation.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -8061,7 +8061,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un slot ; 4 Mio ; même projet/équipe/équipement/véhicule de départ ; commandes visibles en 16:9/mobile ; focus asynchrone gardé par moteur/session ; validation avant mutation.</t>
+          <t xml:space="preserve">Un slot ; 4 Mio ; même projet/équipe/équipement/véhicule de départ ; commandes visibles en 16:9/mobile ; focus sur le résumé avant désactivation, puis restauration gardée par moteur/session ; validation avant mutation.</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">

</xml_diff>